<commit_message>
ecoglobal-105 : Added param passing from category to product, googleanalytic and favicon and data modfied for propbeds
</commit_message>
<xml_diff>
--- a/TODOList.xlsx
+++ b/TODOList.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
   <si>
     <t>Add Minium 10 Category</t>
   </si>
@@ -31,9 +31,6 @@
     <t>Add google Anaytic API key</t>
   </si>
   <si>
-    <t>Sno</t>
-  </si>
-  <si>
     <t>Pass routes from Category to Product</t>
   </si>
   <si>
@@ -65,6 +62,15 @@
   </si>
   <si>
     <t>Host it in Italiy and USA server</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Tasks</t>
   </si>
 </sst>
 </file>
@@ -88,12 +94,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -108,9 +120,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -415,146 +429,158 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="39.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="C4" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="C5" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7">
+      <c r="C6" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11">
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12">
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
         <v>12</v>
       </c>
-      <c r="B13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
         <v>13</v>
       </c>
-      <c r="B14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15">
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
         <v>14</v>
       </c>
-      <c r="B15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16">
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
         <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ecoglobal101 : added feature as category
</commit_message>
<xml_diff>
--- a/TODOList.xlsx
+++ b/TODOList.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
   <si>
     <t>Add Minium 10 Category</t>
   </si>
@@ -43,9 +43,6 @@
     <t>Add Customer Support Boat</t>
   </si>
   <si>
-    <t>Add Contact Us email via mail chimp</t>
-  </si>
-  <si>
     <t>Make About and Services page with images</t>
   </si>
   <si>
@@ -71,6 +68,18 @@
   </si>
   <si>
     <t>Tasks</t>
+  </si>
+  <si>
+    <t>Add Story</t>
+  </si>
+  <si>
+    <t>Add Contact Us email via emailjs</t>
+  </si>
+  <si>
+    <t>Add product section - you will love these</t>
+  </si>
+  <si>
+    <t>Resoruce Library</t>
   </si>
 </sst>
 </file>
@@ -429,7 +438,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="39.85546875" bestFit="1" customWidth="1"/>
@@ -437,10 +446,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -458,6 +467,9 @@
       <c r="B3" t="s">
         <v>1</v>
       </c>
+      <c r="C3" s="2" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
@@ -467,7 +479,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -478,7 +490,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -489,7 +501,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -500,7 +512,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -532,7 +544,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>19</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -540,7 +555,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -548,7 +563,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -556,7 +571,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -564,7 +579,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -572,7 +587,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -580,7 +595,25 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>15</v>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ecoglobal103 : Added Carasoul and featured producted and reduce the size of category images completely
</commit_message>
<xml_diff>
--- a/TODOList.xlsx
+++ b/TODOList.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
   <si>
     <t>Add Minium 10 Category</t>
   </si>
@@ -80,6 +80,15 @@
   </si>
   <si>
     <t>Resoruce Library</t>
+  </si>
+  <si>
+    <t>Fixed Carasoul</t>
+  </si>
+  <si>
+    <t>Fixed Performance issue</t>
+  </si>
+  <si>
+    <t>Remoe Subscribe newsletter</t>
   </si>
 </sst>
 </file>
@@ -438,7 +447,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="39.85546875" bestFit="1" customWidth="1"/>
@@ -459,6 +468,9 @@
       <c r="B2" t="s">
         <v>0</v>
       </c>
+      <c r="C2" s="2" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
@@ -590,7 +602,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -598,7 +610,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -606,14 +618,35 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>